<commit_message>
Finalize internship artifacts and reviewer demo
</commit_message>
<xml_diff>
--- a/Internship_artifacts/Agile_Project_Artifacts_Completed.xlsx
+++ b/Internship_artifacts/Agile_Project_Artifacts_Completed.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R164e1556eb044ade"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Backlog" sheetId="2" r:id="R61b3af50ce1e42d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stand up Meeting" sheetId="3" r:id="R27a76c272e764ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrospection" sheetId="4" r:id="R8f4c087de75e4e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R832a257c5f6e4832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Backlog" sheetId="2" r:id="R7862536482884939"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stand up Meeting" sheetId="3" r:id="R0fa8226bbc9c4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrospection" sheetId="4" r:id="R8271e0efcb7745e8"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="actual" hidden="0" function="0" vbProcedure="0">#REF!</x:definedName>
@@ -1064,7 +1064,7 @@
         <x:v>FastAPI and bcrypt</x:v>
       </x:c>
       <x:c r="G2" s="73" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H2" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1090,7 +1090,7 @@
         <x:v>US-01 and local JSON storage</x:v>
       </x:c>
       <x:c r="G3" s="73" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H3" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1116,7 +1116,7 @@
         <x:v>Document loaders</x:v>
       </x:c>
       <x:c r="G4" s="73" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H4" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1142,7 +1142,7 @@
         <x:v>US-03</x:v>
       </x:c>
       <x:c r="G5" s="73" t="str">
-        <x:v>Full Stack</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H5" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1168,7 +1168,7 @@
         <x:v>US-03</x:v>
       </x:c>
       <x:c r="G6" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H6" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1194,7 +1194,7 @@
         <x:v>US-05 and Gemini API</x:v>
       </x:c>
       <x:c r="G7" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H7" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1220,7 +1220,7 @@
         <x:v>US-03</x:v>
       </x:c>
       <x:c r="G8" s="73" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H8" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1246,7 +1246,7 @@
         <x:v>US-06 and Gemini API</x:v>
       </x:c>
       <x:c r="G9" s="73" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H9" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1272,7 +1272,7 @@
         <x:v>US-02 and analysis results</x:v>
       </x:c>
       <x:c r="G10" s="73" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H10" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1298,7 +1298,7 @@
         <x:v>US-06</x:v>
       </x:c>
       <x:c r="G11" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H11" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1324,7 +1324,7 @@
         <x:v>US-10</x:v>
       </x:c>
       <x:c r="G12" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H12" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1350,7 +1350,7 @@
         <x:v>US-10</x:v>
       </x:c>
       <x:c r="G13" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H13" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1376,7 +1376,7 @@
         <x:v>US-06</x:v>
       </x:c>
       <x:c r="G14" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H14" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1402,7 +1402,7 @@
         <x:v>US-06</x:v>
       </x:c>
       <x:c r="G15" s="73" t="str">
-        <x:v>AI/Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H15" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1428,7 +1428,7 @@
         <x:v>US-14</x:v>
       </x:c>
       <x:c r="G16" s="73" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H16" s="73" t="str">
         <x:v>3- Completed</x:v>
@@ -1454,7 +1454,7 @@
         <x:v>Browser File API and Mammoth</x:v>
       </x:c>
       <x:c r="G17" s="97" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H17" s="97" t="str">
         <x:v>3- Completed</x:v>
@@ -1480,7 +1480,7 @@
         <x:v>US-10</x:v>
       </x:c>
       <x:c r="G18" s="97" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H18" s="97" t="str">
         <x:v>3- Completed</x:v>
@@ -1506,7 +1506,7 @@
         <x:v>US-10</x:v>
       </x:c>
       <x:c r="G19" s="97" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H19" s="97" t="str">
         <x:v>3- Completed</x:v>
@@ -1532,7 +1532,7 @@
         <x:v>Core frontend flows</x:v>
       </x:c>
       <x:c r="G20" s="97" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H20" s="97" t="str">
         <x:v>3- Completed</x:v>
@@ -1558,7 +1558,7 @@
         <x:v>Completed project features</x:v>
       </x:c>
       <x:c r="G21" s="97" t="str">
-        <x:v>Documentation</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H21" s="97" t="str">
         <x:v>3- Completed</x:v>
@@ -1584,7 +1584,7 @@
         <x:v>Google OAuth consent and Gmail API</x:v>
       </x:c>
       <x:c r="G22" s="97" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H22" s="97" t="str">
         <x:v>2- In Progress</x:v>
@@ -1610,7 +1610,7 @@
         <x:v>Responsive UI review</x:v>
       </x:c>
       <x:c r="G23" s="97" t="str">
-        <x:v>Frontend</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H23" s="97" t="str">
         <x:v>2- In Progress</x:v>
@@ -1636,7 +1636,7 @@
         <x:v>Stable API contracts</x:v>
       </x:c>
       <x:c r="G24" s="97" t="str">
-        <x:v>QA</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H24" s="97" t="str">
         <x:v>2- In Progress</x:v>
@@ -1660,7 +1660,7 @@
         <x:v>Docker and cloud account</x:v>
       </x:c>
       <x:c r="G25" s="97" t="str">
-        <x:v>DevOps</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="H25" s="97" t="str">
         <x:v>1- Not Started</x:v>
@@ -1928,7 +1928,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fdbefb5af2c4908"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa207702b00a41f2"/>
 </x:worksheet>
 </file>
 
@@ -2865,7 +2865,7 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="F5" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G5" s="83" t="str">
         <x:v>Build</x:v>
@@ -2910,7 +2910,7 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="F6" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G6" s="83" t="str">
         <x:v>Coding</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="F7" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G7" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3000,7 +3000,7 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="F8" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G8" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3047,7 +3047,7 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="F9" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G9" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3094,7 +3094,7 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="F10" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G10" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3139,7 +3139,7 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="F11" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G11" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3186,7 +3186,7 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="F12" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G12" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3231,7 +3231,7 @@
         <x:v>46265</x:v>
       </x:c>
       <x:c r="F13" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G13" s="83" t="str">
         <x:v>Integration Test</x:v>
@@ -3278,7 +3278,7 @@
         <x:v>46265</x:v>
       </x:c>
       <x:c r="F14" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G14" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3323,7 +3323,7 @@
         <x:v>46267</x:v>
       </x:c>
       <x:c r="F15" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G15" s="83" t="str">
         <x:v>Design</x:v>
@@ -3370,7 +3370,7 @@
         <x:v>46267</x:v>
       </x:c>
       <x:c r="F16" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G16" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3415,7 +3415,7 @@
         <x:v>46267</x:v>
       </x:c>
       <x:c r="F17" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G17" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3460,7 +3460,7 @@
         <x:v>46268</x:v>
       </x:c>
       <x:c r="F18" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G18" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3505,7 +3505,7 @@
         <x:v>46269</x:v>
       </x:c>
       <x:c r="F19" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G19" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3552,7 +3552,7 @@
         <x:v>46269</x:v>
       </x:c>
       <x:c r="F20" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G20" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3597,7 +3597,7 @@
         <x:v>46272</x:v>
       </x:c>
       <x:c r="F21" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G21" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3642,7 +3642,7 @@
         <x:v>46266</x:v>
       </x:c>
       <x:c r="F22" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G22" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3691,7 +3691,7 @@
         <x:v>46273</x:v>
       </x:c>
       <x:c r="F23" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G23" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3738,7 +3738,7 @@
         <x:v>46274</x:v>
       </x:c>
       <x:c r="F24" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G24" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3785,7 +3785,7 @@
         <x:v>46274</x:v>
       </x:c>
       <x:c r="F25" s="77" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G25" s="83" t="str">
         <x:v>Coding</x:v>
@@ -3830,7 +3830,7 @@
         <x:v>46275</x:v>
       </x:c>
       <x:c r="F26" s="82" t="str">
-        <x:v>Project Developer</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="G26" s="83" t="str">
         <x:v>System Test</x:v>
@@ -5055,7 +5055,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47e8bb317205434a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfb7f204c9a495a"/>
 </x:worksheet>
 </file>
 
@@ -5507,7 +5507,7 @@
         <x:v>46269</x:v>
       </x:c>
       <x:c r="E2" s="95" t="str">
-        <x:v>Project Team</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="F2" s="96" t="str">
         <x:v>Validate sample documents early and keep API responses structured.</x:v>
@@ -5784,7 +5784,7 @@
         <x:v>46283</x:v>
       </x:c>
       <x:c r="E3" s="95" t="str">
-        <x:v>Project Team</x:v>
+        <x:v>Param Kumar</x:v>
       </x:c>
       <x:c r="F3" s="96" t="str">
         <x:v>Add evidence and test user-facing failure states before demo.</x:v>

</xml_diff>